<commit_message>
Update munkanaplo.xlsx with new data
</commit_message>
<xml_diff>
--- a/munkanaplo.xlsx
+++ b/munkanaplo.xlsx
@@ -1,98 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\23c-bocskay\Downloads\Botka-Geri--tterem\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB550D09-4D2A-4CCF-A908-7A7A8938DA2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DBE08840-A44D-4C5E-A36E-84C7EC9D15E0}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Munka1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Munka1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Boti csinálta:</t>
-  </si>
-  <si>
-    <t>közösen csináltuk</t>
-  </si>
-  <si>
-    <t>Geri csinálta:</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>Összeg</t>
-  </si>
-  <si>
-    <t>Átlag</t>
-  </si>
-  <si>
-    <t>Göngyölített összeg</t>
-  </si>
-  <si>
-    <t>Darab</t>
-  </si>
-  <si>
-    <t>Oszlop1</t>
-  </si>
-  <si>
-    <t>beosztas+kovetelmenyek fájlrendezés stílus, referencia kiválasztása</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
+      <name val="Calibri"/>
+      <charset val="238"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="238"/>
+      <family val="2"/>
       <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="238"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -184,20 +127,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -205,7 +157,7 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -227,7 +179,7 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -249,7 +201,7 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -271,7 +223,7 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -284,8 +236,8 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="21" formatCode="dd/mmm"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center"/>
+      <border>
         <left/>
         <right style="thin">
           <color indexed="64"/>
@@ -332,25 +284,85 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F1717EB9-1F3D-4F88-9143-59853C691969}" name="Táblázat4" displayName="Táblázat4" ref="A1:D8" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
-  <autoFilter ref="A1:D8" xr:uid="{F1717EB9-1F3D-4F88-9143-59853C691969}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Táblázat4" displayName="Táblázat4" ref="A1:D8" headerRowCount="1" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+  <autoFilter ref="A1:D8"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{5048B36D-790A-49C0-B877-0E806DB4CF85}" name="Oszlop1" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{7EBC6138-26D5-43A6-A795-9908C2268D77}" name="Boti csinálta:" dataDxfId="2" dataCellStyle="Normál"/>
-    <tableColumn id="3" xr3:uid="{AD80EF09-DB6A-4C46-A662-688E412EBBEA}" name="közösen csináltuk" dataDxfId="1" dataCellStyle="Normál"/>
-    <tableColumn id="4" xr3:uid="{1516DAB3-BF48-48B2-A53D-4411BD115266}" name="Geri csinálta:" dataDxfId="0" dataCellStyle="Normál"/>
+    <tableColumn id="1" name="Oszlop1" dataDxfId="4"/>
+    <tableColumn id="2" name="Boti csinálta:" dataDxfId="2" dataCellStyle="Normál"/>
+    <tableColumn id="3" name="közösen csináltuk" dataDxfId="1" dataCellStyle="Normál"/>
+    <tableColumn id="4" name="Geri csinálta:" dataDxfId="0" dataCellStyle="Normál"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -652,94 +664,143 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6794422-089A-4350-9784-308F3A8CCA4D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" customWidth="1"/>
-    <col min="2" max="4" width="48.42578125" customWidth="1"/>
+    <col width="12.42578125" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>2</v>
+    <row r="1" ht="24.75" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Oszlop1</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Boti csinálta:</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>közösen csináltuk</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Geri csinálta:</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2">
+      <c r="A2" s="8" t="n">
         <v>46297</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1"/>
+      <c r="B2" s="9" t="n"/>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>beosztas+kovetelmenyek fájlrendezés stílus, referencia kiválasztása</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="n"/>
     </row>
-    <row r="3" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3" ht="75" customHeight="1">
+      <c r="A3" s="8" t="n">
         <v>46301</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1" t="s">
-        <v>3</v>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>- foglalasok.json adatszerkezetének megtervezése (id, név, email, telefon, dátum, időpont, vendégszám, asztalId, végösszeg, törölt)
+- foglalasok.html és portfolio.html oldalak vázának megtervezése</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row r="4" ht="75" customHeight="1">
+      <c r="A4" s="8" t="n">
         <v>46304</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>- foglalasok.html és portfolio.html létrehozása
+- Navbar és Bootstrap beépítése az összes oldalra, active class javítása
+- foglalasok.json feltöltése 18 előre megadott foglalással</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
     </row>
-    <row r="5" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    <row r="5" ht="75" customHeight="1">
+      <c r="A5" s="8" t="n">
         <v>46308</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>- css/foglalasok.css: Montserrat betűtípus, alap stílus
+- foglalasok.js: foglalások betöltése fetch-csel, táblázat létrehozása JavaScriptből
+- Kártyás nézet JavaScriptből + nézetváltó gombok (Táblázat / Kártya), kártya hover effekt</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n"/>
+      <c r="D5" s="1" t="n"/>
     </row>
-    <row r="6" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="8" t="n">
         <v>46311</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>- Keresés névre és szűrés dátumra
+- „Nincs találat” üzenet, ha nincs megfelelő foglalás
+- Rendezés gombnyomásra (név, dátum, vendégszám, végösszeg; növekvő/csökkenő)</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
     </row>
-    <row r="7" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+    <row r="7" ht="75" customHeight="1">
+      <c r="A7" s="8" t="n">
         <v>46315</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>- Soft delete törlés a táblázatban és a kártyákon (torolt = true), megerősítés + Bootstrap üzenet
+- Fel gomb stílusa (jobb alsó sarok), navbar javítás a portfólión
+- Portfólió oldal: hero fejléc és Rólunk szekció</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n"/>
+      <c r="D7" s="1" t="n"/>
     </row>
-    <row r="8" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
+    <row r="8" ht="75" customHeight="1">
+      <c r="A8" s="10" t="n">
         <v>46318</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>- Portfólió oldal: étlap (hamburgerek, üdítők), nyitvatartás, elérhetőség, footer
+- urlap-validacio.js: űrlap mezőinek ellenőrzése (email, telefon, dátum, foglalt asztal), sikeres foglalás visszajelzése</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n"/>
+      <c r="D8" s="1" t="n"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>